<commit_message>
new branch Negative Testing
</commit_message>
<xml_diff>
--- a/SauceDemoTC&BR.xlsx
+++ b/SauceDemoTC&BR.xlsx
@@ -3960,22 +3960,22 @@
       </c>
     </row>
     <row r="206" spans="1:3">
-      <c r="A206" s="27" t="s">
+      <c r="A206" s="94" t="s">
         <v>126</v>
       </c>
-      <c r="B206" s="41">
+      <c r="B206" s="95">
         <v>18000</v>
       </c>
-      <c r="C206" s="42" t="s">
+      <c r="C206" s="96" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="207" spans="1:3">
-      <c r="A207" s="27" t="s">
+      <c r="A207" s="94" t="s">
         <v>136</v>
       </c>
-      <c r="B207" s="27"/>
-      <c r="C207" s="42" t="s">
+      <c r="B207" s="94"/>
+      <c r="C207" s="96" t="s">
         <v>132</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added CartPage and CartTest classes
</commit_message>
<xml_diff>
--- a/SauceDemoTC&BR.xlsx
+++ b/SauceDemoTC&BR.xlsx
@@ -3960,22 +3960,22 @@
       </c>
     </row>
     <row r="206" spans="1:3">
-      <c r="A206" s="27" t="s">
+      <c r="A206" s="94" t="s">
         <v>126</v>
       </c>
-      <c r="B206" s="41">
+      <c r="B206" s="95">
         <v>18000</v>
       </c>
-      <c r="C206" s="42" t="s">
+      <c r="C206" s="96" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="207" spans="1:3">
-      <c r="A207" s="27" t="s">
+      <c r="A207" s="94" t="s">
         <v>136</v>
       </c>
-      <c r="B207" s="27"/>
-      <c r="C207" s="42" t="s">
+      <c r="B207" s="94"/>
+      <c r="C207" s="96" t="s">
         <v>132</v>
       </c>
     </row>

</xml_diff>